<commit_message>
Daily EOD data and reports for 2026-07-27
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260727.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260727.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.402</v>
+        <v>1.395</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.065</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>4.89%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>214759.76</v>
+        <v>213687.49</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>11029.03</v>
+        <v>9956.76</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.105</v>
+        <v>2.1</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.005</v>
+        <v>-0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>147350</v>
+        <v>147000</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-350</v>
+        <v>-700</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.005</v>
+        <v>1.02</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.035</v>
+        <v>-0.02</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-1.92%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>57745.29</v>
+        <v>58607.16</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-2011.03</v>
+        <v>-1149.16</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>59.75</v>
+        <v>59.8</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>661133.75</v>
+        <v>661687</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>9958.5</v>
+        <v>10511.75</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>132.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-132.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>174.23</v>
+        <v>174.07</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.775</v>
+        <v>0.765</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.295</v>
+        <v>0.285</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>61.46%</t>
+          <t>59.38%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7750</v>
+        <v>7650</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2950</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>115.96</v>
+        <v>116.46</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.74</v>
+        <v>2.24</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.52%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>463840</v>
+        <v>465840</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6960</v>
+        <v>8960</v>
       </c>
     </row>
     <row r="12">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.105</v>
+        <v>-0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-630</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.17</v>
+        <v>37.12</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.5</v>
+        <v>31.36</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.87</v>
+        <v>-1.01</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.69%</t>
+          <t>-3.12%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40572</v>
+        <v>40391.68</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-1120.56</v>
+        <v>-1300.88</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1598903.76</v>
+        <v>1601348.56</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>25253.67</v>
+        <v>27698.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>